<commit_message>
chore(valuation): 밸류에이션 스냅샷 2026-10-18
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/valuation_full.xlsx
+++ b/telegram_research_dashboard/static/valuation_full.xlsx
@@ -815,7 +815,7 @@
         <v>37.73</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>11.7</v>
+        <v>11.58</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>10.05</v>
@@ -847,7 +847,7 @@
         <v>5.72</v>
       </c>
       <c r="U5" s="10" t="n">
-        <v>3.07</v>
+        <v>3.2</v>
       </c>
       <c r="V5" s="10" t="n">
         <v>2.44</v>
@@ -866,7 +866,7 @@
         <v>18.82</v>
       </c>
       <c r="AB5" s="12" t="n">
-        <v>29.54</v>
+        <v>30.55</v>
       </c>
       <c r="AC5" s="12" t="n">
         <v>27.1</v>
@@ -912,7 +912,7 @@
         <v>27.94</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>10.65</v>
+        <v>10.2</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>10.51</v>
@@ -944,7 +944,7 @@
         <v>5.64</v>
       </c>
       <c r="U6" s="10" t="n">
-        <v>2.48</v>
+        <v>2.42</v>
       </c>
       <c r="V6" s="10" t="n">
         <v>2</v>
@@ -963,7 +963,7 @@
         <v>22.59</v>
       </c>
       <c r="AB6" s="12" t="n">
-        <v>26.32</v>
+        <v>27.15</v>
       </c>
       <c r="AC6" s="12" t="n">
         <v>21.08</v>
@@ -1007,7 +1007,7 @@
         <v>37.73</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>15.65</v>
+        <v>17.39</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>10.88</v>
@@ -1039,7 +1039,7 @@
         <v>4.96</v>
       </c>
       <c r="U7" s="10" t="n">
-        <v>3.05</v>
+        <v>3.04</v>
       </c>
       <c r="V7" s="10" t="n">
         <v>2.38</v>
@@ -1058,7 +1058,7 @@
         <v>13.74</v>
       </c>
       <c r="AB7" s="12" t="n">
-        <v>21.59</v>
+        <v>19.97</v>
       </c>
       <c r="AC7" s="12" t="n">
         <v>24.58</v>
@@ -1104,7 +1104,7 @@
         <v>13.27</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>5.11</v>
+        <v>4.73</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>4.38</v>
@@ -1138,7 +1138,7 @@
         <v>2.17</v>
       </c>
       <c r="U8" s="10" t="n">
-        <v>1.15</v>
+        <v>1.23</v>
       </c>
       <c r="V8" s="10" t="n">
         <v>0.95</v>
@@ -1157,7 +1157,7 @@
         <v>17.78</v>
       </c>
       <c r="AB8" s="12" t="n">
-        <v>24.84</v>
+        <v>27.86</v>
       </c>
       <c r="AC8" s="12" t="n">
         <v>23.73</v>
@@ -1199,7 +1199,7 @@
         <v>10.3</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>5.39</v>
+        <v>5.31</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>5.29</v>
@@ -1221,7 +1221,7 @@
         <v>2.35</v>
       </c>
       <c r="U9" s="10" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
       <c r="V9" s="10" t="n">
         <v>0.95</v>
@@ -1240,7 +1240,7 @@
         <v>32.19</v>
       </c>
       <c r="AB9" s="12" t="n">
-        <v>23.73</v>
+        <v>24.44</v>
       </c>
       <c r="AC9" s="12" t="n">
         <v>19.63</v>
@@ -1277,7 +1277,9 @@
       <c r="F10" s="9" t="n">
         <v>36.95</v>
       </c>
-      <c r="G10" s="10" t="n"/>
+      <c r="G10" s="10" t="n">
+        <v>6.37</v>
+      </c>
       <c r="H10" s="10" t="n"/>
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="9" t="n">
@@ -1305,7 +1307,9 @@
       <c r="T10" s="9" t="n">
         <v>2.84</v>
       </c>
-      <c r="U10" s="10" t="n"/>
+      <c r="U10" s="10" t="n">
+        <v>1.46</v>
+      </c>
       <c r="V10" s="10" t="n"/>
       <c r="W10" s="10" t="n"/>
       <c r="X10" s="11" t="n">
@@ -1320,7 +1324,9 @@
       <c r="AA10" s="11" t="n">
         <v>10.15</v>
       </c>
-      <c r="AB10" s="12" t="n"/>
+      <c r="AB10" s="12" t="n">
+        <v>24.85</v>
+      </c>
       <c r="AC10" s="12" t="n"/>
       <c r="AD10" s="12" t="n"/>
       <c r="AE10" s="9" t="n">
@@ -1357,7 +1363,7 @@
         <v>32.18</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>27.64</v>
+        <v>27.15</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>22.6</v>
@@ -1383,7 +1389,7 @@
         <v>10.52</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>9.4</v>
+        <v>9.41</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>7.68</v>
@@ -1402,7 +1408,7 @@
         <v>33.73</v>
       </c>
       <c r="AB11" s="12" t="n">
-        <v>37.42</v>
+        <v>38.12</v>
       </c>
       <c r="AC11" s="12" t="n">
         <v>37.39</v>
@@ -1446,7 +1452,7 @@
         <v>18.39</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>10.98</v>
+        <v>10.88</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>8.19</v>
@@ -1480,7 +1486,7 @@
         <v>6.21</v>
       </c>
       <c r="U12" s="10" t="n">
-        <v>2.26</v>
+        <v>2.66</v>
       </c>
       <c r="V12" s="10" t="n">
         <v>1.77</v>
@@ -1499,7 +1505,7 @@
         <v>41.36</v>
       </c>
       <c r="AB12" s="12" t="n">
-        <v>22.94</v>
+        <v>25.25</v>
       </c>
       <c r="AC12" s="12" t="n">
         <v>24.25</v>
@@ -1543,7 +1549,7 @@
         <v>20.62</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>16.62</v>
+        <v>16.65</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>10.27</v>
@@ -1575,7 +1581,7 @@
         <v>6.44</v>
       </c>
       <c r="U13" s="10" t="n">
-        <v>4.19</v>
+        <v>4.16</v>
       </c>
       <c r="V13" s="10" t="n">
         <v>2.98</v>
@@ -1594,7 +1600,7 @@
         <v>36.6</v>
       </c>
       <c r="AB13" s="12" t="n">
-        <v>28.85</v>
+        <v>28.77</v>
       </c>
       <c r="AC13" s="12" t="n">
         <v>33.88</v>
@@ -1640,7 +1646,7 @@
         <v>14.78</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>7.51</v>
+        <v>7.77</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>6.32</v>
@@ -1674,7 +1680,7 @@
         <v>2.59</v>
       </c>
       <c r="U14" s="10" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="V14" s="10" t="n">
         <v>1.12</v>
@@ -1693,7 +1699,7 @@
         <v>19.3</v>
       </c>
       <c r="AB14" s="12" t="n">
-        <v>18.94</v>
+        <v>18.68</v>
       </c>
       <c r="AC14" s="12" t="n">
         <v>19.16</v>
@@ -1741,7 +1747,7 @@
         <v>13.58</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>5.92</v>
+        <v>5.02</v>
       </c>
       <c r="H15" s="10" t="n">
         <v>4.98</v>
@@ -1775,7 +1781,7 @@
         <v>2.93</v>
       </c>
       <c r="U15" s="10" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="V15" s="10" t="n">
         <v>1.03</v>
@@ -1794,7 +1800,7 @@
         <v>24.23</v>
       </c>
       <c r="AB15" s="12" t="n">
-        <v>24.74</v>
+        <v>29.46</v>
       </c>
       <c r="AC15" s="12" t="n">
         <v>23.13</v>
@@ -2954,7 +2960,7 @@
         <v>20.62</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>10.82</v>
+        <v>10.2</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>9.119999999999999</v>
@@ -2988,7 +2994,7 @@
         <v>4.96</v>
       </c>
       <c r="U32" s="15" t="n">
-        <v>2.37</v>
+        <v>2.42</v>
       </c>
       <c r="V32" s="15" t="n">
         <v>1.89</v>
@@ -3007,7 +3013,7 @@
         <v>22.59</v>
       </c>
       <c r="AB32" s="16" t="n">
-        <v>24.79</v>
+        <v>27.15</v>
       </c>
       <c r="AC32" s="16" t="n">
         <v>23.99</v>
@@ -3538,7 +3544,7 @@
         <v>19.51</v>
       </c>
       <c r="G38" s="15" t="n">
-        <v>13.72</v>
+        <v>12.88</v>
       </c>
       <c r="H38" s="15" t="n">
         <v>10.39</v>
@@ -3576,7 +3582,7 @@
         <v>2.73</v>
       </c>
       <c r="U38" s="15" t="n">
-        <v>2.46</v>
+        <v>2.44</v>
       </c>
       <c r="V38" s="15" t="n">
         <v>1.87</v>
@@ -3597,7 +3603,7 @@
         <v>18.3</v>
       </c>
       <c r="AB38" s="16" t="n">
-        <v>21.59</v>
+        <v>22.2</v>
       </c>
       <c r="AC38" s="16" t="n">
         <v>20.73</v>
@@ -3699,7 +3705,7 @@
         <v>59.99</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>43.17</v>
+        <v>46.33</v>
       </c>
       <c r="H42" s="10" t="n">
         <v>24.08</v>
@@ -3733,7 +3739,7 @@
         <v>6.09</v>
       </c>
       <c r="U42" s="10" t="n">
-        <v>5.26</v>
+        <v>5.2</v>
       </c>
       <c r="V42" s="10" t="n">
         <v>4.54</v>
@@ -3752,7 +3758,7 @@
         <v>10.51</v>
       </c>
       <c r="AB42" s="12" t="n">
-        <v>12.76</v>
+        <v>11.81</v>
       </c>
       <c r="AC42" s="12" t="n">
         <v>20.25</v>
@@ -3800,7 +3806,7 @@
         <v>34.46</v>
       </c>
       <c r="G43" s="10" t="n">
-        <v>19.33</v>
+        <v>20.02</v>
       </c>
       <c r="H43" s="10" t="n">
         <v>15.37</v>
@@ -3834,7 +3840,7 @@
         <v>5</v>
       </c>
       <c r="U43" s="10" t="n">
-        <v>3.92</v>
+        <v>3.74</v>
       </c>
       <c r="V43" s="10" t="n">
         <v>3.24</v>
@@ -3853,7 +3859,7 @@
         <v>19.14</v>
       </c>
       <c r="AB43" s="12" t="n">
-        <v>22.16</v>
+        <v>20.88</v>
       </c>
       <c r="AC43" s="12" t="n">
         <v>23.09</v>
@@ -3901,7 +3907,7 @@
         <v>36.3</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>34.97</v>
+        <v>35.18</v>
       </c>
       <c r="H44" s="10" t="n">
         <v>23.98</v>
@@ -3935,7 +3941,7 @@
         <v>6.43</v>
       </c>
       <c r="U44" s="10" t="n">
-        <v>7.34</v>
+        <v>7.18</v>
       </c>
       <c r="V44" s="10" t="n">
         <v>5.93</v>
@@ -3954,7 +3960,7 @@
         <v>19.2</v>
       </c>
       <c r="AB44" s="12" t="n">
-        <v>22.85</v>
+        <v>22.12</v>
       </c>
       <c r="AC44" s="12" t="n">
         <v>27.37</v>
@@ -4000,7 +4006,7 @@
         <v>41.99</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>76.75</v>
+        <v>109.94</v>
       </c>
       <c r="H45" s="10" t="n">
         <v>34.17</v>
@@ -4034,7 +4040,7 @@
         <v>2.1</v>
       </c>
       <c r="U45" s="10" t="n">
-        <v>2.99</v>
+        <v>2.79</v>
       </c>
       <c r="V45" s="10" t="n">
         <v>2.86</v>
@@ -4053,7 +4059,7 @@
         <v>6.6</v>
       </c>
       <c r="AB45" s="12" t="n">
-        <v>3.93</v>
+        <v>2.68</v>
       </c>
       <c r="AC45" s="12" t="n">
         <v>8.550000000000001</v>
@@ -4101,7 +4107,7 @@
         <v>26.64</v>
       </c>
       <c r="G46" s="10" t="n">
-        <v>12.23</v>
+        <v>12.59</v>
       </c>
       <c r="H46" s="10" t="n">
         <v>9.48</v>
@@ -4135,7 +4141,7 @@
         <v>6.66</v>
       </c>
       <c r="U46" s="10" t="n">
-        <v>2.73</v>
+        <v>2.75</v>
       </c>
       <c r="V46" s="10" t="n">
         <v>2.16</v>
@@ -4154,7 +4160,7 @@
         <v>30.05</v>
       </c>
       <c r="AB46" s="12" t="n">
-        <v>24.88</v>
+        <v>24.25</v>
       </c>
       <c r="AC46" s="12" t="n">
         <v>25.43</v>
@@ -5144,7 +5150,7 @@
         <v>36.3</v>
       </c>
       <c r="G61" s="15" t="n">
-        <v>34.97</v>
+        <v>35.18</v>
       </c>
       <c r="H61" s="15" t="n">
         <v>23.98</v>
@@ -5178,7 +5184,7 @@
         <v>6.09</v>
       </c>
       <c r="U61" s="15" t="n">
-        <v>3.92</v>
+        <v>3.74</v>
       </c>
       <c r="V61" s="15" t="n">
         <v>3.24</v>
@@ -5197,7 +5203,7 @@
         <v>19.14</v>
       </c>
       <c r="AB61" s="16" t="n">
-        <v>22.16</v>
+        <v>20.88</v>
       </c>
       <c r="AC61" s="16" t="n">
         <v>23.09</v>
@@ -5772,7 +5778,7 @@
         <v>4.93</v>
       </c>
       <c r="U67" s="15" t="n">
-        <v>3.84</v>
+        <v>3.75</v>
       </c>
       <c r="V67" s="15" t="n">
         <v>3.35</v>
@@ -5889,7 +5895,7 @@
         <v>47.5</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>7.17</v>
+        <v>7.23</v>
       </c>
       <c r="H71" s="10" t="n">
         <v>6.33</v>
@@ -5923,7 +5929,7 @@
         <v>2.61</v>
       </c>
       <c r="U71" s="10" t="n">
-        <v>1.85</v>
+        <v>0.9</v>
       </c>
       <c r="V71" s="10" t="n">
         <v>1.45</v>
@@ -5942,7 +5948,7 @@
         <v>5.74</v>
       </c>
       <c r="AB71" s="12" t="n">
-        <v>29.37</v>
+        <v>18.21</v>
       </c>
       <c r="AC71" s="12" t="n">
         <v>25.62</v>
@@ -5990,7 +5996,7 @@
         <v>13.73</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>8.32</v>
+        <v>8.75</v>
       </c>
       <c r="H72" s="10" t="n">
         <v>8.140000000000001</v>
@@ -6024,7 +6030,7 @@
         <v>0.77</v>
       </c>
       <c r="U72" s="10" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="V72" s="10" t="n">
         <v>0.61</v>
@@ -6043,7 +6049,7 @@
         <v>5.71</v>
       </c>
       <c r="AB72" s="12" t="n">
-        <v>7.93</v>
+        <v>7.49</v>
       </c>
       <c r="AC72" s="12" t="n">
         <v>7.68</v>
@@ -6172,7 +6178,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>5.56</v>
+        <v>4.21</v>
       </c>
       <c r="H74" s="10" t="n">
         <v>4.57</v>
@@ -6206,7 +6212,7 @@
         <v>0.92</v>
       </c>
       <c r="U74" s="10" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="V74" s="10" t="n">
         <v>0.53</v>
@@ -6225,7 +6231,7 @@
         <v>11.66</v>
       </c>
       <c r="AB74" s="12" t="n">
-        <v>11.18</v>
+        <v>15.39</v>
       </c>
       <c r="AC74" s="12" t="n">
         <v>12.24</v>
@@ -7378,7 +7384,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="G90" s="15" t="n">
-        <v>7.17</v>
+        <v>7.23</v>
       </c>
       <c r="H90" s="15" t="n">
         <v>6.33</v>
@@ -7412,7 +7418,7 @@
         <v>0.66</v>
       </c>
       <c r="U90" s="15" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="V90" s="15" t="n">
         <v>0.61</v>
@@ -7431,7 +7437,7 @@
         <v>7.02</v>
       </c>
       <c r="AB90" s="16" t="n">
-        <v>11.18</v>
+        <v>15.39</v>
       </c>
       <c r="AC90" s="16" t="n">
         <v>12.24</v>
@@ -7911,7 +7917,7 @@
         <v>1.48</v>
       </c>
       <c r="U95" s="15" t="n">
-        <v>1.75</v>
+        <v>1.62</v>
       </c>
       <c r="V95" s="15" t="n">
         <v>1.61</v>
@@ -7932,7 +7938,7 @@
         <v>10.49</v>
       </c>
       <c r="AB95" s="16" t="n">
-        <v>12.16</v>
+        <v>14.02</v>
       </c>
       <c r="AC95" s="16" t="n">
         <v>15.14</v>
@@ -8095,7 +8101,7 @@
         <v>37.73</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>11.7</v>
+        <v>11.58</v>
       </c>
       <c r="K2" s="9" t="n">
         <v>10.05</v>
@@ -8137,7 +8143,7 @@
         <v>27.94</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>10.65</v>
+        <v>10.2</v>
       </c>
       <c r="K3" s="9" t="n">
         <v>10.51</v>
@@ -8177,7 +8183,7 @@
         <v>37.73</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>15.65</v>
+        <v>17.39</v>
       </c>
       <c r="K4" s="9" t="n">
         <v>10.88</v>
@@ -8219,7 +8225,7 @@
         <v>13.27</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>5.11</v>
+        <v>4.73</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>4.38</v>
@@ -8257,7 +8263,7 @@
         <v>10.3</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>5.39</v>
+        <v>5.31</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>5.29</v>
@@ -8296,7 +8302,9 @@
       <c r="I7" s="9" t="n">
         <v>36.95</v>
       </c>
-      <c r="J7" s="9" t="n"/>
+      <c r="J7" s="9" t="n">
+        <v>6.37</v>
+      </c>
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
     </row>
@@ -8803,7 +8811,7 @@
         <v>32.18</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>27.64</v>
+        <v>27.15</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>22.6</v>
@@ -8847,7 +8855,7 @@
         <v>18.39</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>10.98</v>
+        <v>10.88</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>8.19</v>
@@ -8887,7 +8895,7 @@
         <v>20.62</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>16.62</v>
+        <v>16.65</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>10.27</v>
@@ -8929,7 +8937,7 @@
         <v>14.78</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>7.51</v>
+        <v>7.77</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>6.32</v>
@@ -8973,7 +8981,7 @@
         <v>13.58</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>5.92</v>
+        <v>5.02</v>
       </c>
       <c r="K23" s="9" t="n">
         <v>4.98</v>
@@ -9017,7 +9025,7 @@
         <v>59.99</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>43.17</v>
+        <v>46.33</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>24.08</v>
@@ -9061,7 +9069,7 @@
         <v>34.46</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>19.33</v>
+        <v>20.02</v>
       </c>
       <c r="K25" s="9" t="n">
         <v>15.37</v>
@@ -9105,7 +9113,7 @@
         <v>36.3</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>34.97</v>
+        <v>35.18</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>23.98</v>
@@ -9147,7 +9155,7 @@
         <v>41.99</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>76.75</v>
+        <v>109.94</v>
       </c>
       <c r="K27" s="9" t="n">
         <v>34.17</v>
@@ -9191,7 +9199,7 @@
         <v>26.64</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>12.23</v>
+        <v>12.59</v>
       </c>
       <c r="K28" s="9" t="n">
         <v>9.48</v>
@@ -9631,7 +9639,7 @@
         <v>47.5</v>
       </c>
       <c r="J38" s="9" t="n">
-        <v>7.17</v>
+        <v>7.23</v>
       </c>
       <c r="K38" s="9" t="n">
         <v>6.33</v>
@@ -9675,7 +9683,7 @@
         <v>13.73</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>8.32</v>
+        <v>8.75</v>
       </c>
       <c r="K39" s="9" t="n">
         <v>8.140000000000001</v>
@@ -10107,7 +10115,7 @@
         <v>8.390000000000001</v>
       </c>
       <c r="J49" s="9" t="n">
-        <v>5.56</v>
+        <v>4.21</v>
       </c>
       <c r="K49" s="9" t="n">
         <v>4.57</v>
@@ -12473,7 +12481,7 @@
         <v>5.72</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>3.07</v>
+        <v>3.2</v>
       </c>
       <c r="K2" s="9" t="n">
         <v>2.44</v>
@@ -12517,7 +12525,7 @@
         <v>5.64</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>2.48</v>
+        <v>2.42</v>
       </c>
       <c r="K3" s="9" t="n">
         <v>2</v>
@@ -12561,7 +12569,7 @@
         <v>4.96</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>3.05</v>
+        <v>3.04</v>
       </c>
       <c r="K4" s="9" t="n">
         <v>2.38</v>
@@ -12605,7 +12613,7 @@
         <v>2.17</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>1.15</v>
+        <v>1.23</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>0.95</v>
@@ -12643,7 +12651,7 @@
         <v>2.35</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>0.95</v>
@@ -12686,7 +12694,9 @@
       <c r="I7" s="9" t="n">
         <v>2.84</v>
       </c>
-      <c r="J7" s="9" t="n"/>
+      <c r="J7" s="9" t="n">
+        <v>1.46</v>
+      </c>
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
     </row>
@@ -13203,7 +13213,7 @@
         <v>10.52</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>9.4</v>
+        <v>9.41</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>7.68</v>
@@ -13247,7 +13257,7 @@
         <v>6.21</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>2.26</v>
+        <v>2.66</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>1.77</v>
@@ -13291,7 +13301,7 @@
         <v>6.44</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>4.19</v>
+        <v>4.16</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>2.98</v>
@@ -13335,7 +13345,7 @@
         <v>2.59</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>1.12</v>
@@ -13379,7 +13389,7 @@
         <v>2.93</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="K23" s="9" t="n">
         <v>1.03</v>
@@ -13423,7 +13433,7 @@
         <v>6.09</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>5.26</v>
+        <v>5.2</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>4.54</v>
@@ -13467,7 +13477,7 @@
         <v>5</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>3.92</v>
+        <v>3.74</v>
       </c>
       <c r="K25" s="9" t="n">
         <v>3.24</v>
@@ -13511,7 +13521,7 @@
         <v>6.43</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>7.34</v>
+        <v>7.18</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>5.93</v>
@@ -13555,7 +13565,7 @@
         <v>2.1</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>2.99</v>
+        <v>2.79</v>
       </c>
       <c r="K27" s="9" t="n">
         <v>2.86</v>
@@ -13599,7 +13609,7 @@
         <v>6.66</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>2.73</v>
+        <v>2.75</v>
       </c>
       <c r="K28" s="9" t="n">
         <v>2.16</v>
@@ -14039,7 +14049,7 @@
         <v>2.61</v>
       </c>
       <c r="J38" s="9" t="n">
-        <v>1.85</v>
+        <v>0.9</v>
       </c>
       <c r="K38" s="9" t="n">
         <v>1.45</v>
@@ -14083,7 +14093,7 @@
         <v>0.77</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="K39" s="9" t="n">
         <v>0.61</v>
@@ -14519,7 +14529,7 @@
         <v>0.92</v>
       </c>
       <c r="J49" s="9" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K49" s="9" t="n">
         <v>0.53</v>
@@ -14777,7 +14787,7 @@
         <v>18.82</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>29.54</v>
+        <v>30.55</v>
       </c>
       <c r="K2" s="11" t="n">
         <v>27.1</v>
@@ -14821,7 +14831,7 @@
         <v>22.59</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>26.32</v>
+        <v>27.15</v>
       </c>
       <c r="K3" s="11" t="n">
         <v>21.08</v>
@@ -14865,7 +14875,7 @@
         <v>13.74</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>21.59</v>
+        <v>19.97</v>
       </c>
       <c r="K4" s="11" t="n">
         <v>24.58</v>
@@ -14909,7 +14919,7 @@
         <v>17.78</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>24.84</v>
+        <v>27.86</v>
       </c>
       <c r="K5" s="11" t="n">
         <v>23.73</v>
@@ -14953,7 +14963,7 @@
         <v>32.19</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>23.73</v>
+        <v>24.44</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>19.63</v>
@@ -14996,7 +15006,9 @@
       <c r="I7" s="11" t="n">
         <v>10.15</v>
       </c>
-      <c r="J7" s="11" t="n"/>
+      <c r="J7" s="11" t="n">
+        <v>24.85</v>
+      </c>
       <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
     </row>
@@ -15517,7 +15529,7 @@
         <v>33.73</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>37.42</v>
+        <v>38.12</v>
       </c>
       <c r="K19" s="11" t="n">
         <v>37.39</v>
@@ -15561,7 +15573,7 @@
         <v>41.36</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>22.94</v>
+        <v>25.25</v>
       </c>
       <c r="K20" s="11" t="n">
         <v>24.25</v>
@@ -15605,7 +15617,7 @@
         <v>36.6</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>28.85</v>
+        <v>28.77</v>
       </c>
       <c r="K21" s="11" t="n">
         <v>33.88</v>
@@ -15649,7 +15661,7 @@
         <v>19.3</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>18.94</v>
+        <v>18.68</v>
       </c>
       <c r="K22" s="11" t="n">
         <v>19.16</v>
@@ -15693,7 +15705,7 @@
         <v>24.23</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>24.74</v>
+        <v>29.46</v>
       </c>
       <c r="K23" s="11" t="n">
         <v>23.13</v>
@@ -15737,7 +15749,7 @@
         <v>10.51</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>12.76</v>
+        <v>11.81</v>
       </c>
       <c r="K24" s="11" t="n">
         <v>20.25</v>
@@ -15781,7 +15793,7 @@
         <v>19.14</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>22.16</v>
+        <v>20.88</v>
       </c>
       <c r="K25" s="11" t="n">
         <v>23.09</v>
@@ -15825,7 +15837,7 @@
         <v>19.2</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>22.85</v>
+        <v>22.12</v>
       </c>
       <c r="K26" s="11" t="n">
         <v>27.37</v>
@@ -15869,7 +15881,7 @@
         <v>6.6</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>3.93</v>
+        <v>2.68</v>
       </c>
       <c r="K27" s="11" t="n">
         <v>8.550000000000001</v>
@@ -15913,7 +15925,7 @@
         <v>30.05</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>24.88</v>
+        <v>24.25</v>
       </c>
       <c r="K28" s="11" t="n">
         <v>25.43</v>
@@ -16353,7 +16365,7 @@
         <v>5.74</v>
       </c>
       <c r="J38" s="11" t="n">
-        <v>29.37</v>
+        <v>18.21</v>
       </c>
       <c r="K38" s="11" t="n">
         <v>25.62</v>
@@ -16397,7 +16409,7 @@
         <v>5.71</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>7.93</v>
+        <v>7.49</v>
       </c>
       <c r="K39" s="11" t="n">
         <v>7.68</v>
@@ -16833,7 +16845,7 @@
         <v>11.66</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>11.18</v>
+        <v>15.39</v>
       </c>
       <c r="K49" s="11" t="n">
         <v>12.24</v>
@@ -19742,14 +19754,14 @@
         <v>11996718253433.27</v>
       </c>
       <c r="M6" s="17" t="n">
-        <v>11.7</v>
+        <v>11.58</v>
       </c>
       <c r="N6" s="17" t="n"/>
       <c r="O6" s="17" t="n">
-        <v>3.07</v>
+        <v>3.2</v>
       </c>
       <c r="P6" s="17" t="n">
-        <v>29.54</v>
+        <v>30.55</v>
       </c>
       <c r="Q6" s="17" t="n">
         <v>1.49</v>
@@ -20237,14 +20249,14 @@
         <v>8040572283234.132</v>
       </c>
       <c r="M13" s="17" t="n">
-        <v>10.65</v>
+        <v>10.2</v>
       </c>
       <c r="N13" s="17" t="n"/>
       <c r="O13" s="17" t="n">
-        <v>2.48</v>
+        <v>2.42</v>
       </c>
       <c r="P13" s="17" t="n">
-        <v>26.32</v>
+        <v>27.15</v>
       </c>
       <c r="Q13" s="17" t="n">
         <v>1.26</v>
@@ -20730,14 +20742,14 @@
         <v>5153154643491.666</v>
       </c>
       <c r="M20" s="17" t="n">
-        <v>15.65</v>
+        <v>17.39</v>
       </c>
       <c r="N20" s="17" t="n"/>
       <c r="O20" s="17" t="n">
-        <v>3.05</v>
+        <v>3.04</v>
       </c>
       <c r="P20" s="17" t="n">
-        <v>21.59</v>
+        <v>19.97</v>
       </c>
       <c r="Q20" s="17" t="n">
         <v>1.23</v>
@@ -21227,14 +21239,14 @@
         <v>16271603322338.4</v>
       </c>
       <c r="M27" s="17" t="n">
-        <v>5.11</v>
+        <v>4.73</v>
       </c>
       <c r="N27" s="17" t="n"/>
       <c r="O27" s="17" t="n">
-        <v>1.15</v>
+        <v>1.23</v>
       </c>
       <c r="P27" s="17" t="n">
-        <v>24.84</v>
+        <v>27.86</v>
       </c>
       <c r="Q27" s="17" t="n">
         <v>0.54</v>
@@ -21696,14 +21708,14 @@
         <v>1375864481019.893</v>
       </c>
       <c r="M34" s="17" t="n">
-        <v>5.39</v>
+        <v>5.31</v>
       </c>
       <c r="N34" s="17" t="n"/>
       <c r="O34" s="17" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
       <c r="P34" s="17" t="n">
-        <v>23.73</v>
+        <v>24.44</v>
       </c>
       <c r="Q34" s="17" t="n">
         <v>1.18</v>
@@ -22180,10 +22192,16 @@
       </c>
       <c r="K41" s="18" t="n"/>
       <c r="L41" s="18" t="n"/>
-      <c r="M41" s="17" t="n"/>
+      <c r="M41" s="17" t="n">
+        <v>6.37</v>
+      </c>
       <c r="N41" s="17" t="n"/>
-      <c r="O41" s="17" t="n"/>
-      <c r="P41" s="17" t="n"/>
+      <c r="O41" s="17" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="P41" s="17" t="n">
+        <v>24.85</v>
+      </c>
       <c r="Q41" s="17" t="n"/>
       <c r="R41" s="17" t="inlineStr">
         <is>
@@ -28073,14 +28091,14 @@
         <v>1009130437230.669</v>
       </c>
       <c r="M125" s="17" t="n">
-        <v>27.64</v>
+        <v>27.15</v>
       </c>
       <c r="N125" s="17" t="n"/>
       <c r="O125" s="17" t="n">
-        <v>9.4</v>
+        <v>9.41</v>
       </c>
       <c r="P125" s="17" t="n">
-        <v>37.42</v>
+        <v>38.12</v>
       </c>
       <c r="Q125" s="17" t="n">
         <v>3.99</v>
@@ -28572,14 +28590,14 @@
         <v>615574991482</v>
       </c>
       <c r="M132" s="17" t="n">
-        <v>10.98</v>
+        <v>10.88</v>
       </c>
       <c r="N132" s="17" t="n"/>
       <c r="O132" s="17" t="n">
-        <v>2.26</v>
+        <v>2.66</v>
       </c>
       <c r="P132" s="17" t="n">
-        <v>22.94</v>
+        <v>25.25</v>
       </c>
       <c r="Q132" s="17" t="n">
         <v>2.34</v>
@@ -29065,14 +29083,14 @@
         <v>743585229863.8025</v>
       </c>
       <c r="M139" s="17" t="n">
-        <v>16.62</v>
+        <v>16.65</v>
       </c>
       <c r="N139" s="17" t="n"/>
       <c r="O139" s="17" t="n">
-        <v>4.19</v>
+        <v>4.16</v>
       </c>
       <c r="P139" s="17" t="n">
-        <v>28.85</v>
+        <v>28.77</v>
       </c>
       <c r="Q139" s="17" t="n">
         <v>1.98</v>
@@ -29562,14 +29580,14 @@
         <v>680694234169.2651</v>
       </c>
       <c r="M146" s="17" t="n">
-        <v>7.51</v>
+        <v>7.77</v>
       </c>
       <c r="N146" s="17" t="n"/>
       <c r="O146" s="17" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="P146" s="17" t="n">
-        <v>18.94</v>
+        <v>18.68</v>
       </c>
       <c r="Q146" s="17" t="n">
         <v>0.95</v>
@@ -30061,14 +30079,14 @@
         <v>331992443278</v>
       </c>
       <c r="M153" s="17" t="n">
-        <v>5.92</v>
+        <v>5.02</v>
       </c>
       <c r="N153" s="17" t="n"/>
       <c r="O153" s="17" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="P153" s="17" t="n">
-        <v>24.74</v>
+        <v>29.46</v>
       </c>
       <c r="Q153" s="17" t="n">
         <v>0.51</v>
@@ -30560,14 +30578,14 @@
         <v>2007652633721.282</v>
       </c>
       <c r="M160" s="17" t="n">
-        <v>43.17</v>
+        <v>46.33</v>
       </c>
       <c r="N160" s="17" t="n"/>
       <c r="O160" s="17" t="n">
-        <v>5.26</v>
+        <v>5.2</v>
       </c>
       <c r="P160" s="17" t="n">
-        <v>12.76</v>
+        <v>11.81</v>
       </c>
       <c r="Q160" s="17" t="n">
         <v>1.99</v>
@@ -31059,14 +31077,14 @@
         <v>11640307256887.55</v>
       </c>
       <c r="M167" s="17" t="n">
-        <v>19.33</v>
+        <v>20.02</v>
       </c>
       <c r="N167" s="17" t="n"/>
       <c r="O167" s="17" t="n">
-        <v>3.92</v>
+        <v>3.74</v>
       </c>
       <c r="P167" s="17" t="n">
-        <v>22.16</v>
+        <v>20.88</v>
       </c>
       <c r="Q167" s="17" t="n">
         <v>1.42</v>
@@ -31558,14 +31576,14 @@
         <v>1708001170727.462</v>
       </c>
       <c r="M174" s="17" t="n">
-        <v>34.97</v>
+        <v>35.18</v>
       </c>
       <c r="N174" s="17" t="n"/>
       <c r="O174" s="17" t="n">
-        <v>7.34</v>
+        <v>7.18</v>
       </c>
       <c r="P174" s="17" t="n">
-        <v>22.85</v>
+        <v>22.12</v>
       </c>
       <c r="Q174" s="17" t="n">
         <v>2.43</v>
@@ -32055,14 +32073,14 @@
         <v>4946595644964.042</v>
       </c>
       <c r="M181" s="17" t="n">
-        <v>76.75</v>
+        <v>109.94</v>
       </c>
       <c r="N181" s="17" t="n"/>
       <c r="O181" s="17" t="n">
-        <v>2.99</v>
+        <v>2.79</v>
       </c>
       <c r="P181" s="17" t="n">
-        <v>3.93</v>
+        <v>2.68</v>
       </c>
       <c r="Q181" s="17" t="n">
         <v>3.28</v>
@@ -32554,14 +32572,14 @@
         <v>3873726429965.954</v>
       </c>
       <c r="M188" s="17" t="n">
-        <v>12.23</v>
+        <v>12.59</v>
       </c>
       <c r="N188" s="17" t="n"/>
       <c r="O188" s="17" t="n">
-        <v>2.73</v>
+        <v>2.75</v>
       </c>
       <c r="P188" s="17" t="n">
-        <v>24.88</v>
+        <v>24.25</v>
       </c>
       <c r="Q188" s="17" t="n">
         <v>1.57</v>
@@ -37544,14 +37562,14 @@
         <v>2391162650434.556</v>
       </c>
       <c r="M258" s="17" t="n">
-        <v>7.17</v>
+        <v>7.23</v>
       </c>
       <c r="N258" s="17" t="n"/>
       <c r="O258" s="17" t="n">
-        <v>1.85</v>
+        <v>0.9</v>
       </c>
       <c r="P258" s="17" t="n">
-        <v>29.37</v>
+        <v>18.21</v>
       </c>
       <c r="Q258" s="17" t="n">
         <v>0.47</v>
@@ -38043,14 +38061,14 @@
         <v>7585792678930.512</v>
       </c>
       <c r="M265" s="17" t="n">
-        <v>8.32</v>
+        <v>8.75</v>
       </c>
       <c r="N265" s="17" t="n"/>
       <c r="O265" s="17" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="P265" s="17" t="n">
-        <v>7.93</v>
+        <v>7.49</v>
       </c>
       <c r="Q265" s="17" t="n">
         <v>0.51</v>
@@ -42997,14 +43015,14 @@
         <v>328971474869.7184</v>
       </c>
       <c r="M335" s="17" t="n">
-        <v>5.56</v>
+        <v>4.21</v>
       </c>
       <c r="N335" s="17" t="n"/>
       <c r="O335" s="17" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P335" s="17" t="n">
-        <v>11.18</v>
+        <v>15.39</v>
       </c>
       <c r="Q335" s="17" t="n">
         <v>0.38</v>
@@ -44821,7 +44839,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T06:32:46+09:00</t>
+          <t>2026-10-19T06:47:06+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>